<commit_message>
added brandon and ZW validation rules
</commit_message>
<xml_diff>
--- a/Team's_work/Classification of LEA EQA and FOS SSEC 2020 (Latest).xlsx
+++ b/Team's_work/Classification of LEA EQA and FOS SSEC 2020 (Latest).xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3D05CCA8-421E-6C45-87CD-A590EF3CA191}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{643C9260-9601-204F-B5AC-A40840E8F56C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="20740" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Contents" sheetId="7" r:id="rId1"/>
@@ -25,7 +25,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'SSEC2020 (FOS)'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'SSEC2020 (LEA)'!$1:$5</definedName>
   </definedNames>
-  <calcPr calcId="191029" concurrentCalc="0"/>
+  <calcPr calcId="191029" iterate="1" iterateCount="1000" iterateDelta="0.01"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -33,7 +33,12 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -2483,9 +2488,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -2561,12 +2573,15 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -2574,22 +2589,22 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3630,7 +3645,7 @@
       <c r="A29" s="8" t="s">
         <v>720</v>
       </c>
-      <c r="B29" s="8" t="s">
+      <c r="B29" s="10" t="s">
         <v>750</v>
       </c>
     </row>

</xml_diff>